<commit_message>
intermediate step, working on spatial join issues
</commit_message>
<xml_diff>
--- a/data/mining/jasansky/materials_covered.xlsx
+++ b/data/mining/jasansky/materials_covered.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dpsich-my.sharepoint.com/personal/alvaro_hahn-menacho_psi_ch/Documents/Severin's work/4_Github_Repo/semesterproject/data/mining/jasansky/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="11_0E039DCD8F79A8D366075C52F37BD272AA43A735" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1DBA735A-1D18-5EFE-AEA7-456DD024ED72}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="11_0E039DCD8F79A8D366075C52F37BD272AA43A735" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7D92CF6-5A0A-49E4-9DF6-DF7212AE39F1}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="705" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -919,14 +919,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D81"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.58984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -940,7 +941,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -954,7 +955,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -968,7 +969,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -982,7 +983,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -996,7 +997,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1010,7 +1011,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -1024,7 +1025,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -1038,7 +1039,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1052,7 +1053,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -1066,7 +1067,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -1080,7 +1081,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -1094,7 +1095,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A13" t="s">
         <v>4</v>
       </c>
@@ -1108,7 +1109,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -1122,7 +1123,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -1136,7 +1137,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A16" t="s">
         <v>4</v>
       </c>
@@ -1150,7 +1151,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A17" t="s">
         <v>38</v>
       </c>
@@ -1164,7 +1165,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A18" t="s">
         <v>38</v>
       </c>
@@ -1178,7 +1179,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A19" t="s">
         <v>38</v>
       </c>
@@ -1192,7 +1193,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A20" t="s">
         <v>38</v>
       </c>
@@ -1206,7 +1207,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A21" t="s">
         <v>38</v>
       </c>
@@ -1220,7 +1221,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A22" t="s">
         <v>38</v>
       </c>
@@ -1234,7 +1235,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A23" t="s">
         <v>38</v>
       </c>
@@ -1248,7 +1249,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A24" t="s">
         <v>38</v>
       </c>
@@ -1262,7 +1263,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A25" t="s">
         <v>38</v>
       </c>
@@ -1276,7 +1277,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A26" t="s">
         <v>38</v>
       </c>
@@ -1290,7 +1291,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A27" t="s">
         <v>38</v>
       </c>
@@ -1304,7 +1305,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A28" t="s">
         <v>38</v>
       </c>
@@ -1318,7 +1319,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A29" t="s">
         <v>38</v>
       </c>
@@ -1332,7 +1333,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A30" t="s">
         <v>38</v>
       </c>
@@ -1346,7 +1347,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A31" t="s">
         <v>38</v>
       </c>
@@ -1360,7 +1361,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A32" t="s">
         <v>38</v>
       </c>
@@ -1374,7 +1375,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A33" t="s">
         <v>38</v>
       </c>
@@ -1388,7 +1389,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A34" t="s">
         <v>38</v>
       </c>
@@ -1402,7 +1403,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A35" t="s">
         <v>38</v>
       </c>
@@ -1416,7 +1417,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A36" t="s">
         <v>38</v>
       </c>
@@ -1430,7 +1431,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A37" t="s">
         <v>38</v>
       </c>
@@ -1444,7 +1445,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A38" t="s">
         <v>38</v>
       </c>
@@ -1458,7 +1459,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A39" t="s">
         <v>38</v>
       </c>
@@ -1472,7 +1473,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A40" t="s">
         <v>38</v>
       </c>
@@ -1486,7 +1487,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A41" t="s">
         <v>38</v>
       </c>
@@ -1500,7 +1501,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A42" t="s">
         <v>38</v>
       </c>
@@ -1514,7 +1515,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A43" t="s">
         <v>38</v>
       </c>
@@ -1528,7 +1529,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A44" t="s">
         <v>38</v>
       </c>
@@ -1542,7 +1543,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A45" t="s">
         <v>38</v>
       </c>
@@ -1556,7 +1557,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A46" t="s">
         <v>38</v>
       </c>
@@ -1570,7 +1571,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A47" t="s">
         <v>38</v>
       </c>
@@ -1584,7 +1585,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A48" t="s">
         <v>104</v>
       </c>
@@ -1598,7 +1599,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A49" t="s">
         <v>104</v>
       </c>
@@ -1612,7 +1613,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A50" t="s">
         <v>104</v>
       </c>
@@ -1626,7 +1627,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A51" t="s">
         <v>104</v>
       </c>
@@ -1640,7 +1641,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A52" t="s">
         <v>104</v>
       </c>
@@ -1654,7 +1655,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A53" t="s">
         <v>104</v>
       </c>
@@ -1668,7 +1669,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A54" t="s">
         <v>118</v>
       </c>
@@ -1682,7 +1683,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A55" t="s">
         <v>118</v>
       </c>
@@ -1696,7 +1697,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A56" t="s">
         <v>118</v>
       </c>
@@ -1710,7 +1711,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A57" t="s">
         <v>118</v>
       </c>
@@ -1724,7 +1725,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A58" t="s">
         <v>118</v>
       </c>
@@ -1738,7 +1739,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A59" t="s">
         <v>118</v>
       </c>
@@ -1752,7 +1753,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A60" t="s">
         <v>118</v>
       </c>
@@ -1766,7 +1767,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A61" t="s">
         <v>118</v>
       </c>
@@ -1780,7 +1781,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A62" t="s">
         <v>118</v>
       </c>
@@ -1794,7 +1795,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A63" t="s">
         <v>118</v>
       </c>
@@ -1808,7 +1809,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A64" t="s">
         <v>118</v>
       </c>
@@ -1822,7 +1823,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A65" t="s">
         <v>118</v>
       </c>
@@ -1836,7 +1837,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A66" t="s">
         <v>118</v>
       </c>
@@ -1850,7 +1851,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A67" t="s">
         <v>118</v>
       </c>
@@ -1864,7 +1865,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A68" t="s">
         <v>118</v>
       </c>
@@ -1878,7 +1879,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A69" t="s">
         <v>118</v>
       </c>
@@ -1892,7 +1893,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A70" t="s">
         <v>118</v>
       </c>
@@ -1906,7 +1907,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A71" t="s">
         <v>118</v>
       </c>
@@ -1920,7 +1921,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A72" t="s">
         <v>118</v>
       </c>
@@ -1934,7 +1935,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A73" t="s">
         <v>118</v>
       </c>
@@ -1948,7 +1949,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A74" t="s">
         <v>118</v>
       </c>
@@ -1962,7 +1963,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A75" t="s">
         <v>118</v>
       </c>
@@ -1976,7 +1977,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A76" t="s">
         <v>118</v>
       </c>
@@ -1990,7 +1991,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A77" t="s">
         <v>118</v>
       </c>
@@ -2004,7 +2005,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A78" t="s">
         <v>169</v>
       </c>
@@ -2018,7 +2019,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A79" t="s">
         <v>169</v>
       </c>
@@ -2032,7 +2033,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A80" t="s">
         <v>169</v>
       </c>
@@ -2046,7 +2047,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.75">
       <c r="A81" t="s">
         <v>169</v>
       </c>

</xml_diff>